<commit_message>
add demo-temporal and mitigana for time-series and asu testing
</commit_message>
<xml_diff>
--- a/models/demo-hello-world/hello-world.xlsx
+++ b/models/demo-hello-world/hello-world.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/Projects/anse-models/demo-hello-world/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7231F033-CD8C-BA4E-A599-E4826C338C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C2570CC-4D1C-F745-BDAA-38E1ED52B66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="600" windowWidth="25600" windowHeight="26980" activeTab="1" xr2:uid="{73351A0E-E394-C94F-8AB9-3EA9DA143F24}"/>
+    <workbookView xWindow="6840" yWindow="1160" windowWidth="25600" windowHeight="26900" xr2:uid="{73351A0E-E394-C94F-8AB9-3EA9DA143F24}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs - Flow Network" sheetId="1" r:id="rId1"/>
@@ -618,7 +618,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="128">
   <si>
     <t>COMMENT</t>
   </si>
@@ -1405,7 +1405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F935C300-5F44-C54A-ADD4-2A504DCCAD49}">
-  <dimension ref="A1:L112"/>
+  <dimension ref="B1:L112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5703125" defaultRowHeight="16" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
@@ -2168,7 +2168,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="16" customHeight="1">
+    <row r="65" spans="2:8" ht="16" customHeight="1">
       <c r="B65" t="s">
         <v>54</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="16" customHeight="1">
+    <row r="66" spans="2:8" ht="16" customHeight="1">
       <c r="B66" t="s">
         <v>54</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="16" customHeight="1">
+    <row r="67" spans="2:8" ht="16" customHeight="1">
       <c r="B67" t="s">
         <v>54</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="16" customHeight="1">
+    <row r="69" spans="2:8" ht="16" customHeight="1">
       <c r="B69" t="s">
         <v>54</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="16" customHeight="1">
+    <row r="70" spans="2:8" ht="16" customHeight="1">
       <c r="B70" t="s">
         <v>54</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="16" customHeight="1">
+    <row r="71" spans="2:8" ht="16" customHeight="1">
       <c r="B71" t="s">
         <v>54</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="16" customHeight="1">
+    <row r="72" spans="2:8" ht="16" customHeight="1">
       <c r="B72" t="s">
         <v>54</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="16" customHeight="1">
+    <row r="73" spans="2:8" ht="16" customHeight="1">
       <c r="B73" t="s">
         <v>54</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="16" customHeight="1">
+    <row r="74" spans="2:8" ht="16" customHeight="1">
       <c r="B74" t="s">
         <v>54</v>
       </c>
@@ -2339,7 +2339,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:8" s="3" customFormat="1" ht="16" customHeight="1">
+    <row r="76" spans="2:8" s="3" customFormat="1" ht="16" customHeight="1">
       <c r="B76" s="2" t="s">
         <v>55</v>
       </c>
@@ -2362,10 +2362,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="16" customHeight="1">
-      <c r="A78" t="s">
-        <v>0</v>
-      </c>
+    <row r="78" spans="2:8" ht="16" customHeight="1">
       <c r="B78" t="s">
         <v>60</v>
       </c>
@@ -2381,10 +2378,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="16" customHeight="1">
-      <c r="A79" t="s">
-        <v>0</v>
-      </c>
+    <row r="79" spans="2:8" ht="16" customHeight="1">
       <c r="B79" t="s">
         <v>60</v>
       </c>
@@ -2400,10 +2394,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="16" customHeight="1">
-      <c r="A80" t="s">
-        <v>0</v>
-      </c>
+    <row r="80" spans="2:8" ht="16" customHeight="1">
       <c r="B80" t="s">
         <v>60</v>
       </c>
@@ -2419,10 +2410,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="16" customHeight="1">
-      <c r="A81" t="s">
-        <v>0</v>
-      </c>
+    <row r="81" spans="2:10" ht="16" customHeight="1">
       <c r="B81" t="s">
         <v>60</v>
       </c>
@@ -2438,10 +2426,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="16" customHeight="1">
-      <c r="A82" t="s">
-        <v>0</v>
-      </c>
+    <row r="82" spans="2:10" ht="16" customHeight="1">
       <c r="B82" t="s">
         <v>60</v>
       </c>
@@ -2457,10 +2442,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="16" customHeight="1">
-      <c r="A83" t="s">
-        <v>0</v>
-      </c>
+    <row r="83" spans="2:10" ht="16" customHeight="1">
       <c r="B83" t="s">
         <v>60</v>
       </c>
@@ -2476,10 +2458,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="16" customHeight="1">
-      <c r="A84" t="s">
-        <v>0</v>
-      </c>
+    <row r="84" spans="2:10" ht="16" customHeight="1">
       <c r="B84" t="s">
         <v>60</v>
       </c>
@@ -2495,10 +2474,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="16" customHeight="1">
-      <c r="A85" t="s">
-        <v>0</v>
-      </c>
+    <row r="85" spans="2:10" ht="16" customHeight="1">
       <c r="B85" t="s">
         <v>60</v>
       </c>
@@ -2514,7 +2490,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="87" spans="1:10" s="3" customFormat="1" ht="16" customHeight="1">
+    <row r="87" spans="2:10" s="3" customFormat="1" ht="16" customHeight="1">
       <c r="B87" s="2" t="s">
         <v>62</v>
       </c>
@@ -2543,7 +2519,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="16" customHeight="1">
+    <row r="89" spans="2:10" ht="16" customHeight="1">
       <c r="B89" t="s">
         <v>70</v>
       </c>
@@ -2558,7 +2534,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="16" customHeight="1">
+    <row r="90" spans="2:10" ht="16" customHeight="1">
       <c r="B90" t="s">
         <v>70</v>
       </c>
@@ -2573,7 +2549,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="16" customHeight="1">
+    <row r="92" spans="2:10" ht="16" customHeight="1">
       <c r="B92" t="s">
         <v>70</v>
       </c>
@@ -2588,7 +2564,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="16" customHeight="1">
+    <row r="93" spans="2:10" ht="16" customHeight="1">
       <c r="B93" t="s">
         <v>70</v>
       </c>
@@ -2603,7 +2579,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="16" customHeight="1">
+    <row r="95" spans="2:10" ht="16" customHeight="1">
       <c r="B95" t="s">
         <v>70</v>
       </c>
@@ -2618,7 +2594,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="16" customHeight="1">
+    <row r="96" spans="2:10" ht="16" customHeight="1">
       <c r="B96" t="s">
         <v>70</v>
       </c>

</xml_diff>